<commit_message>
Adapt TCL; document TCL and Skyworth
- TCL 50V6EA (ak30a5, Android 9): DeviceProfile entry, TclSource for the
  settings overlay (ShowWindowService), the source provider and the cast
  package; settings entry points route through MainActivity.openPage.
- Accessibility guide copy generalised for sets without an Accessibility
  page; the Skyworth/Coocaa factory-menu steps stay.
- docs/适配/TCL.md and docs/适配/创维.md; the compatibility sheet gains the
  three bench rows (TCL 50V6EA, Skyworth 8R720_A5FP, Skyworth 85A6E).
</commit_message>
<xml_diff>
--- a/docs/机型兼容清单.xlsx
+++ b/docs/机型兼容清单.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'机型清单'!$A$2:$G$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'机型清单'!$A$2:$G$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G160"/>
+  <dimension ref="A1:G163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -443,7 +443,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>共 158 台实测机型。数据来自上游 cleanyourtv/README.md；4.0–5.1 无样本，老设备版的兼容性靠群友实测，不代表已验证。</t>
+          <t>共 161 台实测机型（上游 158 台 + 本机 3 台）。数据来自上游 cleanyourtv/README.md；4.0–5.1 无样本，老设备版的兼容性靠群友实测，不代表已验证。</t>
         </is>
       </c>
     </row>
@@ -6034,8 +6034,119 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>TCL 50V6EA</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>ak30a5, com.tcl.cyberui</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Android 9</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>现代版</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>本机实测 2026-10-26：输入源（sourceprovider）、设置（ShowWindowService）、投屏已适配</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Skyworth</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>8R720_A5FP</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>com.tianci.movieplatform, rootpage.HomeActivity</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Android 13</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>新</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>现代版</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>本机实测 2026-10-23：桌面不声明 CATEGORY_HOME；屏保 com.coocaa.screensaver；设置 com.skyworth.setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Skyworth</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>85A6E</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>8R710_A6E, com.ccos.cooui.movieplatform, movieplatform.MainActivity</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Android 13</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>新</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>现代版</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>本机实测 2026-10-24：桌面类名要认宿主 com.ccos.cooui.movieplatform；没有无障碍设置页，只能用 ADB 开</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:G160"/>
+  <autoFilter ref="A2:G163"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -6115,7 +6226,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -6155,7 +6266,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -6187,7 +6298,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15">
@@ -6229,7 +6340,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20">
@@ -6239,7 +6350,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21">

</xml_diff>